<commit_message>
added gross profit 2nd fix with calcellvalue
</commit_message>
<xml_diff>
--- a/results/carefree_financial.xlsx
+++ b/results/carefree_financial.xlsx
@@ -19474,7 +19474,7 @@
       <c r="L26" s="12">
         <f>400</f>
       </c>
-      <c r="M26" s="19">
+      <c r="M26" s="12">
         <f>400</f>
       </c>
       <c r="N26" s="12">
@@ -19654,7 +19654,7 @@
       <c r="L30" s="12">
         <f>671.99</f>
       </c>
-      <c r="M30" s="12">
+      <c r="M30" s="19">
         <f>1509.94</f>
       </c>
       <c r="N30" s="12">
@@ -20102,7 +20102,7 @@
       <c r="L42" s="12">
         <f>1079.53</f>
       </c>
-      <c r="M42" s="19">
+      <c r="M42" s="12">
         <f>1431.43</f>
       </c>
       <c r="N42" s="12">

</xml_diff>

<commit_message>
added stat reporting to subtext
</commit_message>
<xml_diff>
--- a/results/carefree_financial.xlsx
+++ b/results/carefree_financial.xlsx
@@ -536,7 +536,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -598,16 +598,11 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
-    <border>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
@@ -664,9 +659,6 @@
       <alignment horizontal="right" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
@@ -1192,7 +1184,7 @@
       <c r="L9" s="12">
         <f>62443.29</f>
       </c>
-      <c r="M9" s="21">
+      <c r="M9" s="20">
         <f>25944.2</f>
       </c>
       <c r="N9" s="3"/>
@@ -1294,7 +1286,7 @@
       <c r="L12" s="12">
         <f>0</f>
       </c>
-      <c r="M12" s="21">
+      <c r="M12" s="20">
         <f>0</f>
       </c>
       <c r="N12" s="3"/>
@@ -1396,7 +1388,7 @@
       <c r="L15" s="12">
         <f>42770.82</f>
       </c>
-      <c r="M15" s="22">
+      <c r="M15" s="21">
         <f>39826.63</f>
       </c>
       <c r="N15" s="3"/>
@@ -1540,7 +1532,7 @@
       <c r="L19" s="12">
         <f>K19</f>
       </c>
-      <c r="M19" s="21">
+      <c r="M19" s="20">
         <f>L19</f>
       </c>
       <c r="N19" s="3"/>
@@ -1582,7 +1574,7 @@
       <c r="L20" s="12">
         <f>K20</f>
       </c>
-      <c r="M20" s="21">
+      <c r="M20" s="20">
         <f>L20</f>
       </c>
       <c r="N20" s="3"/>
@@ -1624,7 +1616,7 @@
       <c r="L21" s="12">
         <f>K21</f>
       </c>
-      <c r="M21" s="21">
+      <c r="M21" s="20">
         <f>L21</f>
       </c>
       <c r="N21" s="3"/>
@@ -1666,7 +1658,7 @@
       <c r="L22" s="12">
         <f>K22</f>
       </c>
-      <c r="M22" s="21">
+      <c r="M22" s="20">
         <f>L22</f>
       </c>
       <c r="N22" s="3"/>
@@ -1708,7 +1700,7 @@
       <c r="L23" s="12">
         <f>K23</f>
       </c>
-      <c r="M23" s="21">
+      <c r="M23" s="20">
         <f>L23</f>
       </c>
       <c r="N23" s="3"/>
@@ -1750,7 +1742,7 @@
       <c r="L24" s="12">
         <f>K24</f>
       </c>
-      <c r="M24" s="21">
+      <c r="M24" s="20">
         <f>L24</f>
       </c>
       <c r="N24" s="3"/>
@@ -1792,7 +1784,7 @@
       <c r="L25" s="12">
         <f>-517597.22</f>
       </c>
-      <c r="M25" s="22">
+      <c r="M25" s="21">
         <f>-530560.9</f>
       </c>
       <c r="N25" s="3"/>
@@ -1894,7 +1886,7 @@
       <c r="L28" s="12">
         <f>K28</f>
       </c>
-      <c r="M28" s="21">
+      <c r="M28" s="20">
         <f>L28</f>
       </c>
       <c r="N28" s="3"/>
@@ -1936,7 +1928,7 @@
       <c r="L29" s="12">
         <f>-50388</f>
       </c>
-      <c r="M29" s="21">
+      <c r="M29" s="20">
         <f>-51357</f>
       </c>
       <c r="N29" s="3"/>
@@ -2134,7 +2126,7 @@
       <c r="L36" s="12">
         <f>4555.73</f>
       </c>
-      <c r="M36" s="21">
+      <c r="M36" s="20">
         <f>3149.75</f>
       </c>
       <c r="N36" s="3"/>
@@ -2176,7 +2168,7 @@
       <c r="L37" s="12">
         <f>4121.84</f>
       </c>
-      <c r="M37" s="21">
+      <c r="M37" s="20">
         <f>794.17</f>
       </c>
       <c r="N37" s="3"/>
@@ -2218,7 +2210,7 @@
       <c r="L38" s="12">
         <f>K38</f>
       </c>
-      <c r="M38" s="21">
+      <c r="M38" s="20">
         <f>L38</f>
       </c>
       <c r="N38" s="3"/>
@@ -2260,7 +2252,7 @@
       <c r="L39" s="12">
         <f>7645.52</f>
       </c>
-      <c r="M39" s="21">
+      <c r="M39" s="20">
         <f>2245.52</f>
       </c>
       <c r="N39" s="3"/>
@@ -2302,7 +2294,7 @@
       <c r="L40" s="12">
         <f>7431.36</f>
       </c>
-      <c r="M40" s="21">
+      <c r="M40" s="20">
         <f>7930.81</f>
       </c>
       <c r="N40" s="3"/>
@@ -2386,7 +2378,7 @@
       <c r="L42" s="12">
         <f>452682.67</f>
       </c>
-      <c r="M42" s="21">
+      <c r="M42" s="20">
         <f>442379.08</f>
       </c>
       <c r="N42" s="3"/>
@@ -2428,7 +2420,7 @@
       <c r="L43" s="12">
         <f>K43</f>
       </c>
-      <c r="M43" s="21">
+      <c r="M43" s="20">
         <f>L43</f>
       </c>
       <c r="N43" s="3"/>
@@ -2470,7 +2462,7 @@
       <c r="L44" s="12">
         <f>70450.12</f>
       </c>
-      <c r="M44" s="21">
+      <c r="M44" s="20">
         <f>55668.06</f>
       </c>
       <c r="N44" s="3"/>
@@ -2512,7 +2504,7 @@
       <c r="L45" s="12">
         <f>K45</f>
       </c>
-      <c r="M45" s="21">
+      <c r="M45" s="20">
         <f>L45</f>
       </c>
       <c r="N45" s="3"/>
@@ -2554,7 +2546,7 @@
       <c r="L46" s="12">
         <f>31127.18</f>
       </c>
-      <c r="M46" s="21">
+      <c r="M46" s="20">
         <f>L46</f>
       </c>
       <c r="N46" s="3"/>
@@ -2636,7 +2628,7 @@
       <c r="L48" s="12">
         <f>K48</f>
       </c>
-      <c r="M48" s="21">
+      <c r="M48" s="20">
         <f>L48</f>
       </c>
       <c r="N48" s="3"/>
@@ -2678,7 +2670,7 @@
       <c r="L49" s="12">
         <f>K49</f>
       </c>
-      <c r="M49" s="21">
+      <c r="M49" s="20">
         <f>L49</f>
       </c>
       <c r="N49" s="3"/>
@@ -2720,7 +2712,7 @@
       <c r="L50" s="12">
         <f>K50</f>
       </c>
-      <c r="M50" s="21">
+      <c r="M50" s="20">
         <f>L50</f>
       </c>
       <c r="N50" s="3"/>
@@ -2762,7 +2754,7 @@
       <c r="L51" s="12">
         <f>K51</f>
       </c>
-      <c r="M51" s="21">
+      <c r="M51" s="20">
         <f>L51</f>
       </c>
       <c r="N51" s="3"/>
@@ -2804,7 +2796,7 @@
       <c r="L52" s="12">
         <f>K52</f>
       </c>
-      <c r="M52" s="21">
+      <c r="M52" s="20">
         <f>L52</f>
       </c>
       <c r="N52" s="3"/>
@@ -2846,7 +2838,7 @@
       <c r="L53" s="12">
         <f>K53</f>
       </c>
-      <c r="M53" s="21">
+      <c r="M53" s="20">
         <f>L53</f>
       </c>
       <c r="N53" s="3"/>
@@ -3152,7 +3144,7 @@
       <c r="L61" s="12">
         <f>K61</f>
       </c>
-      <c r="M61" s="21">
+      <c r="M61" s="20">
         <f>L61</f>
       </c>
       <c r="N61" s="3"/>
@@ -3194,7 +3186,7 @@
       <c r="L62" s="12">
         <f>K62</f>
       </c>
-      <c r="M62" s="21">
+      <c r="M62" s="20">
         <f>L62</f>
       </c>
       <c r="N62" s="3"/>
@@ -3236,7 +3228,7 @@
       <c r="L63" s="12">
         <f>K63</f>
       </c>
-      <c r="M63" s="21">
+      <c r="M63" s="20">
         <f>L63</f>
       </c>
       <c r="N63" s="3"/>
@@ -3278,7 +3270,7 @@
       <c r="L64" s="12">
         <f>K64</f>
       </c>
-      <c r="M64" s="21">
+      <c r="M64" s="20">
         <f>L64</f>
       </c>
       <c r="N64" s="3"/>
@@ -3320,7 +3312,7 @@
       <c r="L65" s="12">
         <f>K65</f>
       </c>
-      <c r="M65" s="21">
+      <c r="M65" s="20">
         <f>L65</f>
       </c>
       <c r="N65" s="3"/>
@@ -3586,7 +3578,7 @@
       <c r="L72" s="12">
         <f>K72</f>
       </c>
-      <c r="M72" s="21">
+      <c r="M72" s="20">
         <f>L72</f>
       </c>
       <c r="N72" s="3"/>
@@ -3628,7 +3620,7 @@
       <c r="L73" s="12">
         <f>K73</f>
       </c>
-      <c r="M73" s="21">
+      <c r="M73" s="20">
         <f>L73</f>
       </c>
       <c r="N73" s="3"/>
@@ -3670,7 +3662,7 @@
       <c r="L74" s="12">
         <f>K74</f>
       </c>
-      <c r="M74" s="21">
+      <c r="M74" s="20">
         <f>-21000</f>
       </c>
       <c r="N74" s="3"/>
@@ -3712,7 +3704,7 @@
       <c r="L75" s="12">
         <f>K75</f>
       </c>
-      <c r="M75" s="21">
+      <c r="M75" s="20">
         <f>L75</f>
       </c>
       <c r="N75" s="3"/>
@@ -18697,43 +18689,43 @@
       <c r="O4" s="3"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="24">
+      <c r="B5" s="23">
         <v>23</v>
       </c>
-      <c r="C5" s="24">
+      <c r="C5" s="23">
         <v>20</v>
       </c>
-      <c r="D5" s="24">
+      <c r="D5" s="23">
         <v>21</v>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="23">
         <v>22</v>
       </c>
-      <c r="F5" s="24">
+      <c r="F5" s="23">
         <v>22</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="23">
         <v>21</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="23">
         <v>23</v>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="23">
         <v>21</v>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="23">
         <v>22</v>
       </c>
-      <c r="K5" s="24">
+      <c r="K5" s="23">
         <v>23</v>
       </c>
-      <c r="L5" s="24">
+      <c r="L5" s="23">
         <v>20</v>
       </c>
-      <c r="M5" s="24">
+      <c r="M5" s="23">
         <v>23</v>
       </c>
     </row>
@@ -18836,7 +18828,7 @@
       <c r="L8" s="12">
         <f>50873.19</f>
       </c>
-      <c r="M8" s="12">
+      <c r="M8" s="18">
         <f>52608.83</f>
       </c>
       <c r="N8" s="12">
@@ -18990,7 +18982,7 @@
       <c r="L12" s="12">
         <f>12877</f>
       </c>
-      <c r="M12" s="12">
+      <c r="M12" s="18">
         <f>12770</f>
       </c>
       <c r="N12" s="12">
@@ -19306,7 +19298,7 @@
       <c r="L20" s="13">
         <f>(L10)-(L19)</f>
       </c>
-      <c r="M20" s="20">
+      <c r="M20" s="13">
         <f>(M10)-(M19)</f>
       </c>
       <c r="N20" s="13">
@@ -19490,7 +19482,7 @@
       <c r="L26" s="12">
         <f>400</f>
       </c>
-      <c r="M26" s="12">
+      <c r="M26" s="18">
         <f>400</f>
       </c>
       <c r="N26" s="12">
@@ -19670,7 +19662,7 @@
       <c r="L30" s="12">
         <f>671.99</f>
       </c>
-      <c r="M30" s="18">
+      <c r="M30" s="12">
         <f>1509.94</f>
       </c>
       <c r="N30" s="12">
@@ -19790,7 +19782,7 @@
       <c r="L34" s="12">
         <f>300</f>
       </c>
-      <c r="M34" s="12">
+      <c r="M34" s="18">
         <f>300</f>
       </c>
       <c r="N34" s="12">
@@ -19989,7 +19981,7 @@
       <c r="L39" s="12">
         <f>2669.9</f>
       </c>
-      <c r="M39" s="18">
+      <c r="M39" s="12">
         <f>2669.9</f>
       </c>
       <c r="N39" s="12">
@@ -20073,7 +20065,7 @@
         <f>164.76</f>
       </c>
       <c r="L41" s="12"/>
-      <c r="M41" s="18">
+      <c r="M41" s="12">
         <f>123.19</f>
       </c>
       <c r="N41" s="12">

</xml_diff>

<commit_message>
added red tinting to missing balance sheet items according to workbook
</commit_message>
<xml_diff>
--- a/results/carefree_financial.xlsx
+++ b/results/carefree_financial.xlsx
@@ -508,7 +508,7 @@
       <color/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,8 +535,13 @@
         <fgColor rgb="FF00B050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6600"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -598,11 +603,16 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
@@ -662,6 +672,12 @@
       <alignment horizontal="right" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="right" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="right" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
@@ -1388,7 +1404,7 @@
       <c r="L15" s="12">
         <f>42770.82</f>
       </c>
-      <c r="M15" s="21">
+      <c r="M15" s="23">
         <f>39826.63</f>
       </c>
       <c r="N15" s="3"/>
@@ -1784,7 +1800,7 @@
       <c r="L25" s="12">
         <f>-517597.22</f>
       </c>
-      <c r="M25" s="21">
+      <c r="M25" s="23">
         <f>-530560.9</f>
       </c>
       <c r="N25" s="3"/>
@@ -18689,43 +18705,43 @@
       <c r="O4" s="3"/>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="25">
         <v>23</v>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="25">
         <v>20</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="25">
         <v>21</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="25">
         <v>22</v>
       </c>
-      <c r="F5" s="23">
+      <c r="F5" s="25">
         <v>22</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="25">
         <v>21</v>
       </c>
-      <c r="H5" s="23">
+      <c r="H5" s="25">
         <v>23</v>
       </c>
-      <c r="I5" s="23">
+      <c r="I5" s="25">
         <v>21</v>
       </c>
-      <c r="J5" s="23">
+      <c r="J5" s="25">
         <v>22</v>
       </c>
-      <c r="K5" s="23">
+      <c r="K5" s="25">
         <v>23</v>
       </c>
-      <c r="L5" s="23">
+      <c r="L5" s="25">
         <v>20</v>
       </c>
-      <c r="M5" s="23">
+      <c r="M5" s="25">
         <v>23</v>
       </c>
     </row>
@@ -19208,7 +19224,7 @@
       <c r="L18" s="12">
         <f>7622.43</f>
       </c>
-      <c r="M18" s="12">
+      <c r="M18" s="20">
         <f>9673.11</f>
       </c>
       <c r="N18" s="12">
@@ -19298,7 +19314,7 @@
       <c r="L20" s="13">
         <f>(L10)-(L19)</f>
       </c>
-      <c r="M20" s="13">
+      <c r="M20" s="21">
         <f>(M10)-(M19)</f>
       </c>
       <c r="N20" s="13">
@@ -19383,7 +19399,7 @@
       <c r="L23" s="12">
         <f>5000</f>
       </c>
-      <c r="M23" s="12">
+      <c r="M23" s="20">
         <f>5000</f>
       </c>
       <c r="N23" s="12">
@@ -19482,7 +19498,7 @@
       <c r="L26" s="12">
         <f>400</f>
       </c>
-      <c r="M26" s="18">
+      <c r="M26" s="20">
         <f>400</f>
       </c>
       <c r="N26" s="12">
@@ -19662,7 +19678,7 @@
       <c r="L30" s="12">
         <f>671.99</f>
       </c>
-      <c r="M30" s="12">
+      <c r="M30" s="18">
         <f>1509.94</f>
       </c>
       <c r="N30" s="12">
@@ -19782,7 +19798,7 @@
       <c r="L34" s="12">
         <f>300</f>
       </c>
-      <c r="M34" s="18">
+      <c r="M34" s="20">
         <f>300</f>
       </c>
       <c r="N34" s="12">
@@ -19981,7 +19997,7 @@
       <c r="L39" s="12">
         <f>2669.9</f>
       </c>
-      <c r="M39" s="12">
+      <c r="M39" s="20">
         <f>2669.9</f>
       </c>
       <c r="N39" s="12">
@@ -20026,7 +20042,7 @@
       <c r="L40" s="12">
         <f>2402.07</f>
       </c>
-      <c r="M40" s="12">
+      <c r="M40" s="20">
         <f>2402.07</f>
       </c>
       <c r="N40" s="12">
@@ -20065,7 +20081,7 @@
         <f>164.76</f>
       </c>
       <c r="L41" s="12"/>
-      <c r="M41" s="12">
+      <c r="M41" s="18">
         <f>123.19</f>
       </c>
       <c r="N41" s="12">
@@ -20110,7 +20126,7 @@
       <c r="L42" s="12">
         <f>1079.53</f>
       </c>
-      <c r="M42" s="12">
+      <c r="M42" s="20">
         <f>1431.43</f>
       </c>
       <c r="N42" s="12">
@@ -20153,7 +20169,7 @@
       <c r="L43" s="12">
         <f>9.19</f>
       </c>
-      <c r="M43" s="12">
+      <c r="M43" s="22">
         <f>645.71</f>
       </c>
       <c r="N43" s="12">
@@ -20495,7 +20511,7 @@
       <c r="L53" s="12">
         <f>13932.68</f>
       </c>
-      <c r="M53" s="12">
+      <c r="M53" s="20">
         <f>13932.68</f>
       </c>
       <c r="N53" s="12">

</xml_diff>